<commit_message>
corrections, Suppl Mat, section F
</commit_message>
<xml_diff>
--- a/A_Results_Suppl/Baleen Whale Abundance.xlsx
+++ b/A_Results_Suppl/Baleen Whale Abundance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/86bd8becdb44c660/R-Git projects/WattKrug/A_Results_Suppl/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="8_{2AAD539D-9630-4C8D-A3C8-6FEE3604DC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81CBD69F-5F01-4D9E-AC12-8D02CCB76BFC}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="8_{2AAD539D-9630-4C8D-A3C8-6FEE3604DC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA720964-568C-44E3-BEF4-1FB54C20171B}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="1680" windowWidth="17565" windowHeight="14355" xr2:uid="{AF21E024-BC7E-4352-984F-E68B10625382}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="26970" windowHeight="12945" xr2:uid="{AF21E024-BC7E-4352-984F-E68B10625382}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -525,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82C3B8C9-7696-4D25-8C3E-726728D0E755}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" bestFit="1" customWidth="1"/>
@@ -761,74 +761,77 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14">
-        <v>2000</v>
-      </c>
-      <c r="D14" s="1">
-        <v>1492</v>
-      </c>
-      <c r="E14" t="s">
-        <v>31</v>
-      </c>
-      <c r="F14" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>34</v>
       </c>
       <c r="C15">
+        <v>2000</v>
+      </c>
+      <c r="D15" s="1">
+        <v>1492</v>
+      </c>
+      <c r="E15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16">
         <v>2013</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D16" s="1">
         <f>4898+94</f>
         <v>4992</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E16" t="s">
         <v>35</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F16" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16">
-        <v>2019</v>
-      </c>
-      <c r="D16" s="1">
-        <v>7909</v>
-      </c>
-      <c r="E16" t="s">
-        <v>36</v>
-      </c>
-      <c r="F16" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C17">
         <v>2019</v>
       </c>
       <c r="D17" s="1">
+        <v>7909</v>
+      </c>
+      <c r="E17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18">
+        <v>2019</v>
+      </c>
+      <c r="D18" s="1">
         <v>13486</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E18" t="s">
         <v>38</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F18" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>